<commit_message>
13.10.2026 - Update GoLive
</commit_message>
<xml_diff>
--- a/daten/Zoopedia_PZ2_Daten.xlsx
+++ b/daten/Zoopedia_PZ2_Daten.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alle Tiere" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inhalte" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiernamen" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abweichungen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiernamen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abweichungen" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Alle Tiere'!$A$4:$CZ$140</definedName>
@@ -113,7 +114,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -212,11 +213,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -286,6 +327,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -952,80 +1003,80 @@
           <t>Gehegeart</t>
         </is>
       </c>
-      <c r="K1" s="4" t="n"/>
-      <c r="L1" s="4" t="n"/>
-      <c r="M1" s="4" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="28" t="n"/>
       <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Ökologische Rolle(n)</t>
         </is>
       </c>
-      <c r="O1" s="4" t="n"/>
-      <c r="P1" s="4" t="n"/>
-      <c r="Q1" s="4" t="n"/>
-      <c r="R1" s="4" t="n"/>
-      <c r="S1" s="4" t="n"/>
-      <c r="T1" s="4" t="n"/>
-      <c r="U1" s="4" t="n"/>
-      <c r="V1" s="4" t="n"/>
-      <c r="W1" s="4" t="n"/>
-      <c r="X1" s="4" t="n"/>
-      <c r="Y1" s="4" t="n"/>
-      <c r="Z1" s="4" t="n"/>
-      <c r="AA1" s="4" t="n"/>
-      <c r="AB1" s="4" t="n"/>
-      <c r="AC1" s="4" t="n"/>
-      <c r="AD1" s="4" t="n"/>
-      <c r="AE1" s="4" t="n"/>
-      <c r="AF1" s="4" t="n"/>
-      <c r="AG1" s="4" t="n"/>
-      <c r="AH1" s="4" t="n"/>
-      <c r="AI1" s="4" t="n"/>
-      <c r="AJ1" s="4" t="n"/>
+      <c r="O1" s="27" t="n"/>
+      <c r="P1" s="27" t="n"/>
+      <c r="Q1" s="27" t="n"/>
+      <c r="R1" s="27" t="n"/>
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="27" t="n"/>
+      <c r="U1" s="27" t="n"/>
+      <c r="V1" s="27" t="n"/>
+      <c r="W1" s="27" t="n"/>
+      <c r="X1" s="27" t="n"/>
+      <c r="Y1" s="27" t="n"/>
+      <c r="Z1" s="27" t="n"/>
+      <c r="AA1" s="27" t="n"/>
+      <c r="AB1" s="27" t="n"/>
+      <c r="AC1" s="27" t="n"/>
+      <c r="AD1" s="27" t="n"/>
+      <c r="AE1" s="27" t="n"/>
+      <c r="AF1" s="27" t="n"/>
+      <c r="AG1" s="27" t="n"/>
+      <c r="AH1" s="27" t="n"/>
+      <c r="AI1" s="27" t="n"/>
+      <c r="AJ1" s="28" t="n"/>
       <c r="AK1" s="4" t="inlineStr">
         <is>
           <t>Kontinente / Ozeane</t>
         </is>
       </c>
-      <c r="AL1" s="4" t="n"/>
-      <c r="AM1" s="4" t="n"/>
-      <c r="AN1" s="4" t="n"/>
-      <c r="AO1" s="4" t="n"/>
-      <c r="AP1" s="4" t="n"/>
-      <c r="AQ1" s="4" t="n"/>
-      <c r="AR1" s="4" t="n"/>
-      <c r="AS1" s="4" t="n"/>
-      <c r="AT1" s="4" t="n"/>
-      <c r="AU1" s="4" t="n"/>
-      <c r="AV1" s="4" t="n"/>
+      <c r="AL1" s="27" t="n"/>
+      <c r="AM1" s="27" t="n"/>
+      <c r="AN1" s="27" t="n"/>
+      <c r="AO1" s="27" t="n"/>
+      <c r="AP1" s="27" t="n"/>
+      <c r="AQ1" s="27" t="n"/>
+      <c r="AR1" s="27" t="n"/>
+      <c r="AS1" s="27" t="n"/>
+      <c r="AT1" s="27" t="n"/>
+      <c r="AU1" s="27" t="n"/>
+      <c r="AV1" s="28" t="n"/>
       <c r="AW1" s="4" t="inlineStr">
         <is>
           <t>Biome</t>
         </is>
       </c>
-      <c r="AX1" s="4" t="n"/>
-      <c r="AY1" s="4" t="n"/>
-      <c r="AZ1" s="4" t="n"/>
-      <c r="BA1" s="4" t="n"/>
-      <c r="BB1" s="4" t="n"/>
-      <c r="BC1" s="4" t="n"/>
-      <c r="BD1" s="4" t="n"/>
-      <c r="BE1" s="4" t="n"/>
-      <c r="BF1" s="4" t="n"/>
-      <c r="BG1" s="4" t="n"/>
-      <c r="BH1" s="4" t="n"/>
+      <c r="AX1" s="27" t="n"/>
+      <c r="AY1" s="27" t="n"/>
+      <c r="AZ1" s="27" t="n"/>
+      <c r="BA1" s="27" t="n"/>
+      <c r="BB1" s="27" t="n"/>
+      <c r="BC1" s="27" t="n"/>
+      <c r="BD1" s="27" t="n"/>
+      <c r="BE1" s="27" t="n"/>
+      <c r="BF1" s="27" t="n"/>
+      <c r="BG1" s="27" t="n"/>
+      <c r="BH1" s="28" t="n"/>
       <c r="BI1" s="4" t="inlineStr">
         <is>
           <t>Temperatur</t>
         </is>
       </c>
-      <c r="BJ1" s="4" t="n"/>
+      <c r="BJ1" s="28" t="n"/>
       <c r="BK1" s="4" t="inlineStr">
         <is>
           <t>Luftfeuchtigkeit</t>
         </is>
       </c>
-      <c r="BL1" s="4" t="n"/>
+      <c r="BL1" s="28" t="n"/>
       <c r="BM1" s="4" t="inlineStr">
         <is>
           <t>Salzgehalt</t>
@@ -1037,188 +1088,188 @@
 (Fläche jeweils je 1 ausgewachsenes Tier)</t>
         </is>
       </c>
-      <c r="BO1" s="4" t="n"/>
-      <c r="BP1" s="4" t="n"/>
-      <c r="BQ1" s="4" t="n"/>
-      <c r="BR1" s="4" t="n"/>
-      <c r="BS1" s="4" t="n"/>
+      <c r="BO1" s="27" t="n"/>
+      <c r="BP1" s="27" t="n"/>
+      <c r="BQ1" s="27" t="n"/>
+      <c r="BR1" s="27" t="n"/>
+      <c r="BS1" s="28" t="n"/>
       <c r="BT1" s="4" t="inlineStr">
         <is>
           <t>Minimale Gehegevoraussetzungen
 (Fläche jeweils je 2 ausgewachsene Tiere)</t>
         </is>
       </c>
-      <c r="BU1" s="4" t="n"/>
-      <c r="BV1" s="4" t="n"/>
-      <c r="BW1" s="4" t="n"/>
-      <c r="BX1" s="4" t="n"/>
-      <c r="BY1" s="4" t="n"/>
+      <c r="BU1" s="27" t="n"/>
+      <c r="BV1" s="27" t="n"/>
+      <c r="BW1" s="27" t="n"/>
+      <c r="BX1" s="27" t="n"/>
+      <c r="BY1" s="28" t="n"/>
       <c r="BZ1" s="5" t="inlineStr">
         <is>
           <t>Wert, um den es sich pro weiterem
 ausgewachsenen Tier erhöht</t>
         </is>
       </c>
-      <c r="CA1" s="5" t="n"/>
-      <c r="CB1" s="5" t="n"/>
-      <c r="CC1" s="5" t="n"/>
-      <c r="CD1" s="5" t="n"/>
-      <c r="CE1" s="5" t="n"/>
+      <c r="CA1" s="27" t="n"/>
+      <c r="CB1" s="27" t="n"/>
+      <c r="CC1" s="27" t="n"/>
+      <c r="CD1" s="27" t="n"/>
+      <c r="CE1" s="28" t="n"/>
       <c r="CF1" s="4" t="inlineStr">
         <is>
           <t>Zaunanforderungen</t>
         </is>
       </c>
-      <c r="CG1" s="4" t="n"/>
-      <c r="CH1" s="4" t="n"/>
-      <c r="CI1" s="4" t="n"/>
-      <c r="CJ1" s="4" t="n"/>
-      <c r="CK1" s="4" t="n"/>
+      <c r="CG1" s="27" t="n"/>
+      <c r="CH1" s="27" t="n"/>
+      <c r="CI1" s="27" t="n"/>
+      <c r="CJ1" s="27" t="n"/>
+      <c r="CK1" s="28" t="n"/>
       <c r="CL1" s="4" t="inlineStr">
         <is>
           <t>Sozialverhalten</t>
         </is>
       </c>
-      <c r="CM1" s="4" t="n"/>
-      <c r="CN1" s="4" t="n"/>
-      <c r="CO1" s="4" t="n"/>
-      <c r="CP1" s="4" t="n"/>
-      <c r="CQ1" s="4" t="n"/>
-      <c r="CR1" s="4" t="n"/>
+      <c r="CM1" s="27" t="n"/>
+      <c r="CN1" s="27" t="n"/>
+      <c r="CO1" s="27" t="n"/>
+      <c r="CP1" s="27" t="n"/>
+      <c r="CQ1" s="27" t="n"/>
+      <c r="CR1" s="28" t="n"/>
       <c r="CS1" s="4" t="inlineStr">
         <is>
           <t>Lebenszyklus</t>
         </is>
       </c>
-      <c r="CT1" s="4" t="n"/>
-      <c r="CU1" s="4" t="n"/>
-      <c r="CV1" s="4" t="n"/>
-      <c r="CW1" s="4" t="n"/>
+      <c r="CT1" s="27" t="n"/>
+      <c r="CU1" s="27" t="n"/>
+      <c r="CV1" s="27" t="n"/>
+      <c r="CW1" s="28" t="n"/>
       <c r="CX1" s="4" t="inlineStr">
         <is>
           <t>Zusammenleben-
 Option</t>
         </is>
       </c>
-      <c r="CY1" s="4" t="n"/>
-      <c r="CZ1" s="4" t="n"/>
+      <c r="CY1" s="27" t="n"/>
+      <c r="CZ1" s="28" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n"/>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-      <c r="Z2" s="4" t="n"/>
-      <c r="AA2" s="4" t="n"/>
-      <c r="AB2" s="4" t="n"/>
-      <c r="AC2" s="4" t="n"/>
-      <c r="AD2" s="4" t="n"/>
-      <c r="AE2" s="4" t="n"/>
-      <c r="AF2" s="4" t="n"/>
-      <c r="AG2" s="4" t="n"/>
-      <c r="AH2" s="4" t="n"/>
-      <c r="AI2" s="4" t="n"/>
-      <c r="AJ2" s="4" t="n"/>
-      <c r="AK2" s="4" t="n"/>
-      <c r="AL2" s="4" t="n"/>
-      <c r="AM2" s="4" t="n"/>
-      <c r="AN2" s="4" t="n"/>
-      <c r="AO2" s="4" t="n"/>
-      <c r="AP2" s="4" t="n"/>
-      <c r="AQ2" s="4" t="n"/>
-      <c r="AR2" s="4" t="n"/>
-      <c r="AS2" s="4" t="n"/>
-      <c r="AT2" s="4" t="n"/>
-      <c r="AU2" s="4" t="n"/>
-      <c r="AV2" s="4" t="n"/>
-      <c r="AW2" s="4" t="n"/>
-      <c r="AX2" s="4" t="n"/>
-      <c r="AY2" s="4" t="n"/>
-      <c r="AZ2" s="4" t="n"/>
-      <c r="BA2" s="4" t="n"/>
-      <c r="BB2" s="4" t="n"/>
-      <c r="BC2" s="4" t="n"/>
-      <c r="BD2" s="4" t="n"/>
-      <c r="BE2" s="4" t="n"/>
-      <c r="BF2" s="4" t="n"/>
-      <c r="BG2" s="4" t="n"/>
-      <c r="BH2" s="4" t="n"/>
-      <c r="BI2" s="4" t="n"/>
-      <c r="BJ2" s="4" t="n"/>
-      <c r="BK2" s="4" t="n"/>
-      <c r="BL2" s="4" t="n"/>
-      <c r="BM2" s="4" t="n"/>
-      <c r="BN2" s="4" t="n"/>
-      <c r="BO2" s="4" t="n"/>
-      <c r="BP2" s="4" t="n"/>
-      <c r="BQ2" s="4" t="n"/>
-      <c r="BR2" s="4" t="n"/>
-      <c r="BS2" s="4" t="n"/>
-      <c r="BT2" s="4" t="n"/>
-      <c r="BU2" s="4" t="n"/>
-      <c r="BV2" s="4" t="n"/>
-      <c r="BW2" s="4" t="n"/>
-      <c r="BX2" s="4" t="n"/>
-      <c r="BY2" s="4" t="n"/>
-      <c r="BZ2" s="5" t="n"/>
-      <c r="CA2" s="5" t="n"/>
-      <c r="CB2" s="5" t="n"/>
-      <c r="CC2" s="5" t="n"/>
-      <c r="CD2" s="5" t="n"/>
-      <c r="CE2" s="5" t="n"/>
-      <c r="CF2" s="4" t="n"/>
-      <c r="CG2" s="4" t="n"/>
-      <c r="CH2" s="4" t="n"/>
-      <c r="CI2" s="4" t="n"/>
-      <c r="CJ2" s="4" t="n"/>
-      <c r="CK2" s="4" t="n"/>
-      <c r="CL2" s="4" t="n"/>
-      <c r="CM2" s="4" t="n"/>
-      <c r="CN2" s="4" t="n"/>
-      <c r="CO2" s="4" t="n"/>
-      <c r="CP2" s="4" t="n"/>
-      <c r="CQ2" s="4" t="n"/>
-      <c r="CR2" s="4" t="n"/>
-      <c r="CS2" s="4" t="n"/>
-      <c r="CT2" s="4" t="n"/>
-      <c r="CU2" s="4" t="n"/>
-      <c r="CV2" s="4" t="n"/>
-      <c r="CW2" s="4" t="n"/>
-      <c r="CX2" s="4" t="n"/>
-      <c r="CY2" s="4" t="n"/>
-      <c r="CZ2" s="4" t="n"/>
+      <c r="A2" s="29" t="n"/>
+      <c r="B2" s="29" t="n"/>
+      <c r="C2" s="29" t="n"/>
+      <c r="D2" s="29" t="n"/>
+      <c r="E2" s="29" t="n"/>
+      <c r="F2" s="29" t="n"/>
+      <c r="G2" s="29" t="n"/>
+      <c r="H2" s="29" t="n"/>
+      <c r="I2" s="29" t="n"/>
+      <c r="J2" s="30" t="n"/>
+      <c r="K2" s="31" t="n"/>
+      <c r="L2" s="31" t="n"/>
+      <c r="M2" s="32" t="n"/>
+      <c r="N2" s="30" t="n"/>
+      <c r="O2" s="31" t="n"/>
+      <c r="P2" s="31" t="n"/>
+      <c r="Q2" s="31" t="n"/>
+      <c r="R2" s="31" t="n"/>
+      <c r="S2" s="31" t="n"/>
+      <c r="T2" s="31" t="n"/>
+      <c r="U2" s="31" t="n"/>
+      <c r="V2" s="31" t="n"/>
+      <c r="W2" s="31" t="n"/>
+      <c r="X2" s="31" t="n"/>
+      <c r="Y2" s="31" t="n"/>
+      <c r="Z2" s="31" t="n"/>
+      <c r="AA2" s="31" t="n"/>
+      <c r="AB2" s="31" t="n"/>
+      <c r="AC2" s="31" t="n"/>
+      <c r="AD2" s="31" t="n"/>
+      <c r="AE2" s="31" t="n"/>
+      <c r="AF2" s="31" t="n"/>
+      <c r="AG2" s="31" t="n"/>
+      <c r="AH2" s="31" t="n"/>
+      <c r="AI2" s="31" t="n"/>
+      <c r="AJ2" s="32" t="n"/>
+      <c r="AK2" s="30" t="n"/>
+      <c r="AL2" s="31" t="n"/>
+      <c r="AM2" s="31" t="n"/>
+      <c r="AN2" s="31" t="n"/>
+      <c r="AO2" s="31" t="n"/>
+      <c r="AP2" s="31" t="n"/>
+      <c r="AQ2" s="31" t="n"/>
+      <c r="AR2" s="31" t="n"/>
+      <c r="AS2" s="31" t="n"/>
+      <c r="AT2" s="31" t="n"/>
+      <c r="AU2" s="31" t="n"/>
+      <c r="AV2" s="32" t="n"/>
+      <c r="AW2" s="30" t="n"/>
+      <c r="AX2" s="31" t="n"/>
+      <c r="AY2" s="31" t="n"/>
+      <c r="AZ2" s="31" t="n"/>
+      <c r="BA2" s="31" t="n"/>
+      <c r="BB2" s="31" t="n"/>
+      <c r="BC2" s="31" t="n"/>
+      <c r="BD2" s="31" t="n"/>
+      <c r="BE2" s="31" t="n"/>
+      <c r="BF2" s="31" t="n"/>
+      <c r="BG2" s="31" t="n"/>
+      <c r="BH2" s="32" t="n"/>
+      <c r="BI2" s="30" t="n"/>
+      <c r="BJ2" s="32" t="n"/>
+      <c r="BK2" s="30" t="n"/>
+      <c r="BL2" s="32" t="n"/>
+      <c r="BM2" s="29" t="n"/>
+      <c r="BN2" s="30" t="n"/>
+      <c r="BO2" s="31" t="n"/>
+      <c r="BP2" s="31" t="n"/>
+      <c r="BQ2" s="31" t="n"/>
+      <c r="BR2" s="31" t="n"/>
+      <c r="BS2" s="32" t="n"/>
+      <c r="BT2" s="30" t="n"/>
+      <c r="BU2" s="31" t="n"/>
+      <c r="BV2" s="31" t="n"/>
+      <c r="BW2" s="31" t="n"/>
+      <c r="BX2" s="31" t="n"/>
+      <c r="BY2" s="32" t="n"/>
+      <c r="BZ2" s="30" t="n"/>
+      <c r="CA2" s="31" t="n"/>
+      <c r="CB2" s="31" t="n"/>
+      <c r="CC2" s="31" t="n"/>
+      <c r="CD2" s="31" t="n"/>
+      <c r="CE2" s="32" t="n"/>
+      <c r="CF2" s="30" t="n"/>
+      <c r="CG2" s="31" t="n"/>
+      <c r="CH2" s="31" t="n"/>
+      <c r="CI2" s="31" t="n"/>
+      <c r="CJ2" s="31" t="n"/>
+      <c r="CK2" s="32" t="n"/>
+      <c r="CL2" s="30" t="n"/>
+      <c r="CM2" s="31" t="n"/>
+      <c r="CN2" s="31" t="n"/>
+      <c r="CO2" s="31" t="n"/>
+      <c r="CP2" s="31" t="n"/>
+      <c r="CQ2" s="31" t="n"/>
+      <c r="CR2" s="32" t="n"/>
+      <c r="CS2" s="30" t="n"/>
+      <c r="CT2" s="31" t="n"/>
+      <c r="CU2" s="31" t="n"/>
+      <c r="CV2" s="31" t="n"/>
+      <c r="CW2" s="32" t="n"/>
+      <c r="CX2" s="30" t="n"/>
+      <c r="CY2" s="31" t="n"/>
+      <c r="CZ2" s="32" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="29" t="n"/>
+      <c r="B3" s="29" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="29" t="n"/>
+      <c r="E3" s="29" t="n"/>
+      <c r="F3" s="29" t="n"/>
+      <c r="G3" s="29" t="n"/>
+      <c r="H3" s="29" t="n"/>
+      <c r="I3" s="29" t="n"/>
       <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Gehege
@@ -1404,7 +1455,7 @@
           <t>bis</t>
         </is>
       </c>
-      <c r="BM3" s="6" t="n"/>
+      <c r="BM3" s="29" t="n"/>
       <c r="BN3" s="10" t="inlineStr">
         <is>
           <t>Rückzugs-ort</t>
@@ -1515,8 +1566,8 @@
           <t>Wassergraben als Zaun</t>
         </is>
       </c>
-      <c r="CJ3" s="12" t="n"/>
-      <c r="CK3" s="13" t="n"/>
+      <c r="CJ3" s="33" t="n"/>
+      <c r="CK3" s="34" t="n"/>
       <c r="CL3" s="10" t="inlineStr">
         <is>
           <t>Gemischt MIN</t>
@@ -1532,7 +1583,7 @@
           <t>Gemischt Verhältnis</t>
         </is>
       </c>
-      <c r="CO3" s="13" t="n"/>
+      <c r="CO3" s="34" t="n"/>
       <c r="CP3" s="10" t="inlineStr">
         <is>
           <t>Nur
@@ -1594,15 +1645,15 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="A4" s="15" t="n"/>
+      <c r="B4" s="15" t="n"/>
+      <c r="C4" s="15" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="15" t="n"/>
+      <c r="G4" s="15" t="n"/>
+      <c r="H4" s="15" t="n"/>
+      <c r="I4" s="15" t="n"/>
       <c r="J4" s="15" t="n"/>
       <c r="K4" s="15" t="n"/>
       <c r="L4" s="15" t="n"/>
@@ -1771,7 +1822,7 @@
       <c r="BJ4" s="15" t="n"/>
       <c r="BK4" s="15" t="n"/>
       <c r="BL4" s="15" t="n"/>
-      <c r="BM4" s="6" t="n"/>
+      <c r="BM4" s="15" t="n"/>
       <c r="BN4" s="15" t="n"/>
       <c r="BO4" s="15" t="n"/>
       <c r="BP4" s="15" t="n"/>
@@ -36995,8 +37046,8 @@
     <mergeCell ref="CV3:CV4"/>
     <mergeCell ref="CX3:CX4"/>
     <mergeCell ref="AK3:AK4"/>
+    <mergeCell ref="AW3:AW4"/>
     <mergeCell ref="C1:C4"/>
-    <mergeCell ref="AW3:AW4"/>
     <mergeCell ref="BT3:BT4"/>
     <mergeCell ref="E1:E4"/>
     <mergeCell ref="BA3:BA4"/>
@@ -37211,14 +37262,74 @@
           <t>Nein</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4515760/Planet_Zoo_2_Deluxe_Upgrade_Pack/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>Angabe</t>
+        </is>
+      </c>
+      <c r="B1" s="35" t="inlineStr">
+        <is>
+          <t>Wert</t>
+        </is>
+      </c>
+      <c r="C1" s="35" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B2" s="36" t="inlineStr">
+        <is>
+          <t>1.0.3.1011968</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Wird auf der Webseite oben links unter „Zoopedia“ angezeigt. Bei neuer Version hier ändern.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48490,7 +48601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>